<commit_message>
feat: add water service lab prompts and simplify learner folders
</commit_message>
<xml_diff>
--- a/labs/lab-01-excel-to-word/data/Northstar_Work_Orders.xlsx
+++ b/labs/lab-01-excel-to-word/data/Northstar_Work_Orders.xlsx
@@ -510,7 +510,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>Northstar Facilities - fictional</t>
+          <t>Northstar Water Services - fictional water-pipe maintenance and service company</t>
         </is>
       </c>
     </row>
@@ -670,7 +670,7 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
@@ -708,7 +708,7 @@
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 001</t>
+          <t>Leak Repair scheduled or reactive task 001</t>
         </is>
       </c>
     </row>
@@ -725,7 +725,7 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
@@ -763,7 +763,7 @@
       </c>
       <c r="M3" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 002</t>
+          <t>Leak Repair scheduled or reactive task 002</t>
         </is>
       </c>
     </row>
@@ -780,7 +780,7 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
@@ -816,7 +816,7 @@
       </c>
       <c r="M4" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 003</t>
+          <t>Leak Repair scheduled or reactive task 003</t>
         </is>
       </c>
     </row>
@@ -833,7 +833,7 @@
       </c>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve"> hvac </t>
+          <t xml:space="preserve"> Leak repair </t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
@@ -869,7 +869,7 @@
       </c>
       <c r="M5" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 004</t>
+          <t>Leak Repair scheduled or reactive task 004</t>
         </is>
       </c>
     </row>
@@ -886,7 +886,7 @@
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
@@ -922,7 +922,7 @@
       </c>
       <c r="M6" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 005</t>
+          <t>Valve Repair scheduled or reactive task 005</t>
         </is>
       </c>
     </row>
@@ -939,7 +939,7 @@
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
@@ -977,7 +977,7 @@
       </c>
       <c r="M7" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 006</t>
+          <t>Valve Repair scheduled or reactive task 006</t>
         </is>
       </c>
     </row>
@@ -994,7 +994,7 @@
       </c>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -1032,7 +1032,7 @@
       </c>
       <c r="M8" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 007</t>
+          <t>Valve Repair scheduled or reactive task 007</t>
         </is>
       </c>
     </row>
@@ -1049,7 +1049,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
@@ -1085,7 +1085,7 @@
       </c>
       <c r="M9" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 008</t>
+          <t>Valve Repair scheduled or reactive task 008</t>
         </is>
       </c>
     </row>
@@ -1102,7 +1102,7 @@
       </c>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
@@ -1138,7 +1138,7 @@
       </c>
       <c r="M10" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 009</t>
+          <t>Pipe Replacement scheduled or reactive task 009</t>
         </is>
       </c>
     </row>
@@ -1155,7 +1155,7 @@
       </c>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
@@ -1191,7 +1191,7 @@
       </c>
       <c r="M11" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 010</t>
+          <t>Pipe Replacement scheduled or reactive task 010</t>
         </is>
       </c>
     </row>
@@ -1208,7 +1208,7 @@
       </c>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
@@ -1246,7 +1246,7 @@
       </c>
       <c r="M12" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 011</t>
+          <t>Pipe Replacement scheduled or reactive task 011</t>
         </is>
       </c>
     </row>
@@ -1263,7 +1263,7 @@
       </c>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="M13" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 012</t>
+          <t>Pipe Replacement scheduled or reactive task 012</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t xml:space="preserve">Fire safety </t>
+          <t xml:space="preserve">Pump service </t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
@@ -1350,7 +1350,7 @@
       </c>
       <c r="M14" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 013</t>
+          <t>Pump Service scheduled or reactive task 013</t>
         </is>
       </c>
     </row>
@@ -1367,7 +1367,7 @@
       </c>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
@@ -1403,7 +1403,7 @@
       </c>
       <c r="M15" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 014</t>
+          <t>Pump Service scheduled or reactive task 014</t>
         </is>
       </c>
     </row>
@@ -1420,7 +1420,7 @@
       </c>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
@@ -1456,7 +1456,7 @@
       </c>
       <c r="M16" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 015</t>
+          <t>Pump Service scheduled or reactive task 015</t>
         </is>
       </c>
     </row>
@@ -1473,7 +1473,7 @@
       </c>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="M17" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 016</t>
+          <t>Pump Service scheduled or reactive task 016</t>
         </is>
       </c>
     </row>
@@ -1528,7 +1528,7 @@
       </c>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
@@ -1566,7 +1566,7 @@
       </c>
       <c r="M18" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 017</t>
+          <t>Meter Service scheduled or reactive task 017</t>
         </is>
       </c>
     </row>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
@@ -1619,7 +1619,7 @@
       </c>
       <c r="M19" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 018</t>
+          <t>Meter Service scheduled or reactive task 018</t>
         </is>
       </c>
     </row>
@@ -1636,7 +1636,7 @@
       </c>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
@@ -1672,7 +1672,7 @@
       </c>
       <c r="M20" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 019</t>
+          <t>Meter Service scheduled or reactive task 019</t>
         </is>
       </c>
     </row>
@@ -1689,7 +1689,7 @@
       </c>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
@@ -1725,7 +1725,7 @@
       </c>
       <c r="M21" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 020</t>
+          <t>Meter Service scheduled or reactive task 020</t>
         </is>
       </c>
     </row>
@@ -1742,7 +1742,7 @@
       </c>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1780,7 +1780,7 @@
       </c>
       <c r="M22" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 021</t>
+          <t>Leak Repair scheduled or reactive task 021</t>
         </is>
       </c>
     </row>
@@ -1797,7 +1797,7 @@
       </c>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
@@ -1835,7 +1835,7 @@
       </c>
       <c r="M23" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 022</t>
+          <t>Leak Repair scheduled or reactive task 022</t>
         </is>
       </c>
     </row>
@@ -1852,7 +1852,7 @@
       </c>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
@@ -1888,7 +1888,7 @@
       </c>
       <c r="M24" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 023</t>
+          <t>Leak Repair scheduled or reactive task 023</t>
         </is>
       </c>
     </row>
@@ -1905,7 +1905,7 @@
       </c>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
@@ -1941,7 +1941,7 @@
       </c>
       <c r="M25" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 024</t>
+          <t>Leak Repair scheduled or reactive task 024</t>
         </is>
       </c>
     </row>
@@ -1958,7 +1958,7 @@
       </c>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
@@ -1990,7 +1990,7 @@
       </c>
       <c r="M26" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 025</t>
+          <t>Valve Repair scheduled or reactive task 025</t>
         </is>
       </c>
     </row>
@@ -2007,7 +2007,7 @@
       </c>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
@@ -2045,7 +2045,7 @@
       </c>
       <c r="M27" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 026</t>
+          <t>Valve Repair scheduled or reactive task 026</t>
         </is>
       </c>
     </row>
@@ -2062,7 +2062,7 @@
       </c>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
@@ -2100,7 +2100,7 @@
       </c>
       <c r="M28" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 027</t>
+          <t>Valve Repair scheduled or reactive task 027</t>
         </is>
       </c>
     </row>
@@ -2117,7 +2117,7 @@
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
@@ -2153,7 +2153,7 @@
       </c>
       <c r="M29" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 028</t>
+          <t>Valve Repair scheduled or reactive task 028</t>
         </is>
       </c>
     </row>
@@ -2170,7 +2170,7 @@
       </c>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
@@ -2206,7 +2206,7 @@
       </c>
       <c r="M30" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 029</t>
+          <t>Pipe Replacement scheduled or reactive task 029</t>
         </is>
       </c>
     </row>
@@ -2223,7 +2223,7 @@
       </c>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
@@ -2259,7 +2259,7 @@
       </c>
       <c r="M31" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 030</t>
+          <t>Pipe Replacement scheduled or reactive task 030</t>
         </is>
       </c>
     </row>
@@ -2276,7 +2276,7 @@
       </c>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2314,7 +2314,7 @@
       </c>
       <c r="M32" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 031</t>
+          <t>Pipe Replacement scheduled or reactive task 031</t>
         </is>
       </c>
     </row>
@@ -2331,7 +2331,7 @@
       </c>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
@@ -2369,7 +2369,7 @@
       </c>
       <c r="M33" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 032</t>
+          <t>Pipe Replacement scheduled or reactive task 032</t>
         </is>
       </c>
     </row>
@@ -2386,7 +2386,7 @@
       </c>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
@@ -2422,7 +2422,7 @@
       </c>
       <c r="M34" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 033</t>
+          <t>Pump Service scheduled or reactive task 033</t>
         </is>
       </c>
     </row>
@@ -2439,7 +2439,7 @@
       </c>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
@@ -2475,7 +2475,7 @@
       </c>
       <c r="M35" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 034</t>
+          <t>Pump Service scheduled or reactive task 034</t>
         </is>
       </c>
     </row>
@@ -2492,7 +2492,7 @@
       </c>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
@@ -2528,7 +2528,7 @@
       </c>
       <c r="M36" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 035</t>
+          <t>Pump Service scheduled or reactive task 035</t>
         </is>
       </c>
     </row>
@@ -2545,7 +2545,7 @@
       </c>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
@@ -2583,7 +2583,7 @@
       </c>
       <c r="M37" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 036</t>
+          <t>Pump Service scheduled or reactive task 036</t>
         </is>
       </c>
     </row>
@@ -2600,7 +2600,7 @@
       </c>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
@@ -2638,7 +2638,7 @@
       </c>
       <c r="M38" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 037</t>
+          <t>Meter Service scheduled or reactive task 037</t>
         </is>
       </c>
     </row>
@@ -2655,7 +2655,7 @@
       </c>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
@@ -2691,7 +2691,7 @@
       </c>
       <c r="M39" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 038</t>
+          <t>Meter Service scheduled or reactive task 038</t>
         </is>
       </c>
     </row>
@@ -2708,7 +2708,7 @@
       </c>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
@@ -2744,7 +2744,7 @@
       </c>
       <c r="M40" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 039</t>
+          <t>Meter Service scheduled or reactive task 039</t>
         </is>
       </c>
     </row>
@@ -2761,7 +2761,7 @@
       </c>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
@@ -2797,7 +2797,7 @@
       </c>
       <c r="M41" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 040</t>
+          <t>Meter Service scheduled or reactive task 040</t>
         </is>
       </c>
     </row>
@@ -2814,7 +2814,7 @@
       </c>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
@@ -2852,7 +2852,7 @@
       </c>
       <c r="M42" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 041</t>
+          <t>Leak Repair scheduled or reactive task 041</t>
         </is>
       </c>
     </row>
@@ -2869,7 +2869,7 @@
       </c>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
@@ -2907,7 +2907,7 @@
       </c>
       <c r="M43" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 042</t>
+          <t>Leak Repair scheduled or reactive task 042</t>
         </is>
       </c>
     </row>
@@ -2924,7 +2924,7 @@
       </c>
       <c r="C44" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D44" s="2" t="inlineStr">
@@ -2960,7 +2960,7 @@
       </c>
       <c r="M44" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 043</t>
+          <t>Leak Repair scheduled or reactive task 043</t>
         </is>
       </c>
     </row>
@@ -2977,7 +2977,7 @@
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D45" s="2" t="inlineStr">
@@ -3013,7 +3013,7 @@
       </c>
       <c r="M45" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 044</t>
+          <t>Leak Repair scheduled or reactive task 044</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D46" s="2" t="inlineStr">
@@ -3066,7 +3066,7 @@
       </c>
       <c r="M46" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 045</t>
+          <t>Valve Repair scheduled or reactive task 045</t>
         </is>
       </c>
     </row>
@@ -3083,7 +3083,7 @@
       </c>
       <c r="C47" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D47" s="2" t="inlineStr">
@@ -3121,7 +3121,7 @@
       </c>
       <c r="M47" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 046</t>
+          <t>Valve Repair scheduled or reactive task 046</t>
         </is>
       </c>
     </row>
@@ -3138,7 +3138,7 @@
       </c>
       <c r="C48" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D48" s="2" t="inlineStr">
@@ -3176,7 +3176,7 @@
       </c>
       <c r="M48" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 047</t>
+          <t>Valve Repair scheduled or reactive task 047</t>
         </is>
       </c>
     </row>
@@ -3193,7 +3193,7 @@
       </c>
       <c r="C49" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D49" s="2" t="inlineStr">
@@ -3229,7 +3229,7 @@
       </c>
       <c r="M49" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 048</t>
+          <t>Valve Repair scheduled or reactive task 048</t>
         </is>
       </c>
     </row>
@@ -3246,7 +3246,7 @@
       </c>
       <c r="C50" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D50" s="2" t="inlineStr">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="M50" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 049</t>
+          <t>Pipe Replacement scheduled or reactive task 049</t>
         </is>
       </c>
     </row>
@@ -3295,7 +3295,7 @@
       </c>
       <c r="C51" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D51" s="2" t="inlineStr">
@@ -3331,7 +3331,7 @@
       </c>
       <c r="M51" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 050</t>
+          <t>Pipe Replacement scheduled or reactive task 050</t>
         </is>
       </c>
     </row>
@@ -3348,7 +3348,7 @@
       </c>
       <c r="C52" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D52" s="2" t="inlineStr">
@@ -3386,7 +3386,7 @@
       </c>
       <c r="M52" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 051</t>
+          <t>Pipe Replacement scheduled or reactive task 051</t>
         </is>
       </c>
     </row>
@@ -3403,7 +3403,7 @@
       </c>
       <c r="C53" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D53" s="2" t="inlineStr">
@@ -3441,7 +3441,7 @@
       </c>
       <c r="M53" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 052</t>
+          <t>Pipe Replacement scheduled or reactive task 052</t>
         </is>
       </c>
     </row>
@@ -3458,7 +3458,7 @@
       </c>
       <c r="C54" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D54" s="2" t="inlineStr">
@@ -3494,7 +3494,7 @@
       </c>
       <c r="M54" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 053</t>
+          <t>Pump Service scheduled or reactive task 053</t>
         </is>
       </c>
     </row>
@@ -3511,7 +3511,7 @@
       </c>
       <c r="C55" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D55" s="2" t="inlineStr">
@@ -3547,7 +3547,7 @@
       </c>
       <c r="M55" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 054</t>
+          <t>Pump Service scheduled or reactive task 054</t>
         </is>
       </c>
     </row>
@@ -3564,7 +3564,7 @@
       </c>
       <c r="C56" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D56" s="2" t="inlineStr">
@@ -3600,7 +3600,7 @@
       </c>
       <c r="M56" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 055</t>
+          <t>Pump Service scheduled or reactive task 055</t>
         </is>
       </c>
     </row>
@@ -3617,7 +3617,7 @@
       </c>
       <c r="C57" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D57" s="2" t="inlineStr">
@@ -3655,7 +3655,7 @@
       </c>
       <c r="M57" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 056</t>
+          <t>Pump Service scheduled or reactive task 056</t>
         </is>
       </c>
     </row>
@@ -3672,7 +3672,7 @@
       </c>
       <c r="C58" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D58" s="2" t="inlineStr">
@@ -3710,7 +3710,7 @@
       </c>
       <c r="M58" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 057</t>
+          <t>Meter Service scheduled or reactive task 057</t>
         </is>
       </c>
     </row>
@@ -3727,7 +3727,7 @@
       </c>
       <c r="C59" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D59" s="2" t="inlineStr">
@@ -3763,7 +3763,7 @@
       </c>
       <c r="M59" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 058</t>
+          <t>Meter Service scheduled or reactive task 058</t>
         </is>
       </c>
     </row>
@@ -3780,7 +3780,7 @@
       </c>
       <c r="C60" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D60" s="2" t="inlineStr">
@@ -3816,7 +3816,7 @@
       </c>
       <c r="M60" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 059</t>
+          <t>Meter Service scheduled or reactive task 059</t>
         </is>
       </c>
     </row>
@@ -3833,7 +3833,7 @@
       </c>
       <c r="C61" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D61" s="2" t="inlineStr">
@@ -3869,7 +3869,7 @@
       </c>
       <c r="M61" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 060</t>
+          <t>Meter Service scheduled or reactive task 060</t>
         </is>
       </c>
     </row>
@@ -3886,7 +3886,7 @@
       </c>
       <c r="C62" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D62" s="2" t="inlineStr">
@@ -3924,7 +3924,7 @@
       </c>
       <c r="M62" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 061</t>
+          <t>Leak Repair scheduled or reactive task 061</t>
         </is>
       </c>
     </row>
@@ -3941,7 +3941,7 @@
       </c>
       <c r="C63" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D63" s="2" t="inlineStr">
@@ -3979,7 +3979,7 @@
       </c>
       <c r="M63" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 062</t>
+          <t>Leak Repair scheduled or reactive task 062</t>
         </is>
       </c>
     </row>
@@ -3996,7 +3996,7 @@
       </c>
       <c r="C64" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D64" s="2" t="inlineStr">
@@ -4032,7 +4032,7 @@
       </c>
       <c r="M64" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 063</t>
+          <t>Leak Repair scheduled or reactive task 063</t>
         </is>
       </c>
     </row>
@@ -4049,7 +4049,7 @@
       </c>
       <c r="C65" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D65" s="2" t="inlineStr">
@@ -4085,7 +4085,7 @@
       </c>
       <c r="M65" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 064</t>
+          <t>Leak Repair scheduled or reactive task 064</t>
         </is>
       </c>
     </row>
@@ -4102,7 +4102,7 @@
       </c>
       <c r="C66" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D66" s="2" t="inlineStr">
@@ -4138,7 +4138,7 @@
       </c>
       <c r="M66" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 065</t>
+          <t>Valve Repair scheduled or reactive task 065</t>
         </is>
       </c>
     </row>
@@ -4155,7 +4155,7 @@
       </c>
       <c r="C67" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D67" s="2" t="inlineStr">
@@ -4193,7 +4193,7 @@
       </c>
       <c r="M67" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 066</t>
+          <t>Valve Repair scheduled or reactive task 066</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="C68" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D68" s="2" t="inlineStr">
@@ -4248,7 +4248,7 @@
       </c>
       <c r="M68" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 067</t>
+          <t>Valve Repair scheduled or reactive task 067</t>
         </is>
       </c>
     </row>
@@ -4265,7 +4265,7 @@
       </c>
       <c r="C69" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D69" s="2" t="inlineStr">
@@ -4301,7 +4301,7 @@
       </c>
       <c r="M69" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 068</t>
+          <t>Valve Repair scheduled or reactive task 068</t>
         </is>
       </c>
     </row>
@@ -4318,7 +4318,7 @@
       </c>
       <c r="C70" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D70" s="2" t="inlineStr">
@@ -4354,7 +4354,7 @@
       </c>
       <c r="M70" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 069</t>
+          <t>Pipe Replacement scheduled or reactive task 069</t>
         </is>
       </c>
     </row>
@@ -4371,7 +4371,7 @@
       </c>
       <c r="C71" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D71" s="2" t="inlineStr">
@@ -4407,7 +4407,7 @@
       </c>
       <c r="M71" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 070</t>
+          <t>Pipe Replacement scheduled or reactive task 070</t>
         </is>
       </c>
     </row>
@@ -4424,7 +4424,7 @@
       </c>
       <c r="C72" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D72" s="2" t="inlineStr">
@@ -4462,7 +4462,7 @@
       </c>
       <c r="M72" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 071</t>
+          <t>Pipe Replacement scheduled or reactive task 071</t>
         </is>
       </c>
     </row>
@@ -4479,7 +4479,7 @@
       </c>
       <c r="C73" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D73" s="2" t="inlineStr">
@@ -4517,7 +4517,7 @@
       </c>
       <c r="M73" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 072</t>
+          <t>Pipe Replacement scheduled or reactive task 072</t>
         </is>
       </c>
     </row>
@@ -4534,7 +4534,7 @@
       </c>
       <c r="C74" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D74" s="2" t="inlineStr">
@@ -4566,7 +4566,7 @@
       </c>
       <c r="M74" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 073</t>
+          <t>Pump Service scheduled or reactive task 073</t>
         </is>
       </c>
     </row>
@@ -4583,7 +4583,7 @@
       </c>
       <c r="C75" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D75" s="2" t="inlineStr">
@@ -4619,7 +4619,7 @@
       </c>
       <c r="M75" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 074</t>
+          <t>Pump Service scheduled or reactive task 074</t>
         </is>
       </c>
     </row>
@@ -4636,7 +4636,7 @@
       </c>
       <c r="C76" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D76" s="2" t="inlineStr">
@@ -4672,7 +4672,7 @@
       </c>
       <c r="M76" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 075</t>
+          <t>Pump Service scheduled or reactive task 075</t>
         </is>
       </c>
     </row>
@@ -4689,7 +4689,7 @@
       </c>
       <c r="C77" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D77" s="2" t="inlineStr">
@@ -4727,7 +4727,7 @@
       </c>
       <c r="M77" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 076</t>
+          <t>Pump Service scheduled or reactive task 076</t>
         </is>
       </c>
     </row>
@@ -4744,7 +4744,7 @@
       </c>
       <c r="C78" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D78" s="2" t="inlineStr">
@@ -4782,7 +4782,7 @@
       </c>
       <c r="M78" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 077</t>
+          <t>Meter Service scheduled or reactive task 077</t>
         </is>
       </c>
     </row>
@@ -4799,7 +4799,7 @@
       </c>
       <c r="C79" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D79" s="2" t="inlineStr">
@@ -4835,7 +4835,7 @@
       </c>
       <c r="M79" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 078</t>
+          <t>Meter Service scheduled or reactive task 078</t>
         </is>
       </c>
     </row>
@@ -4852,7 +4852,7 @@
       </c>
       <c r="C80" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D80" s="2" t="inlineStr">
@@ -4888,7 +4888,7 @@
       </c>
       <c r="M80" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 079</t>
+          <t>Meter Service scheduled or reactive task 079</t>
         </is>
       </c>
     </row>
@@ -4905,7 +4905,7 @@
       </c>
       <c r="C81" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D81" s="2" t="inlineStr">
@@ -4941,7 +4941,7 @@
       </c>
       <c r="M81" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 080</t>
+          <t>Meter Service scheduled or reactive task 080</t>
         </is>
       </c>
     </row>
@@ -4958,7 +4958,7 @@
       </c>
       <c r="C82" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D82" s="2" t="inlineStr">
@@ -4996,7 +4996,7 @@
       </c>
       <c r="M82" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 081</t>
+          <t>Leak Repair scheduled or reactive task 081</t>
         </is>
       </c>
     </row>
@@ -5013,7 +5013,7 @@
       </c>
       <c r="C83" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D83" s="2" t="inlineStr">
@@ -5051,7 +5051,7 @@
       </c>
       <c r="M83" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 082</t>
+          <t>Leak Repair scheduled or reactive task 082</t>
         </is>
       </c>
     </row>
@@ -5068,7 +5068,7 @@
       </c>
       <c r="C84" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D84" s="2" t="inlineStr">
@@ -5104,7 +5104,7 @@
       </c>
       <c r="M84" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 083</t>
+          <t>Leak Repair scheduled or reactive task 083</t>
         </is>
       </c>
     </row>
@@ -5121,7 +5121,7 @@
       </c>
       <c r="C85" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D85" s="2" t="inlineStr">
@@ -5157,7 +5157,7 @@
       </c>
       <c r="M85" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 084</t>
+          <t>Leak Repair scheduled or reactive task 084</t>
         </is>
       </c>
     </row>
@@ -5174,7 +5174,7 @@
       </c>
       <c r="C86" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D86" s="2" t="inlineStr">
@@ -5206,7 +5206,7 @@
       </c>
       <c r="M86" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 085</t>
+          <t>Valve Repair scheduled or reactive task 085</t>
         </is>
       </c>
     </row>
@@ -5223,7 +5223,7 @@
       </c>
       <c r="C87" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D87" s="2" t="inlineStr">
@@ -5261,7 +5261,7 @@
       </c>
       <c r="M87" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 086</t>
+          <t>Valve Repair scheduled or reactive task 086</t>
         </is>
       </c>
     </row>
@@ -5278,7 +5278,7 @@
       </c>
       <c r="C88" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D88" s="2" t="inlineStr">
@@ -5316,7 +5316,7 @@
       </c>
       <c r="M88" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 087</t>
+          <t>Valve Repair scheduled or reactive task 087</t>
         </is>
       </c>
     </row>
@@ -5333,7 +5333,7 @@
       </c>
       <c r="C89" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D89" s="2" t="inlineStr">
@@ -5369,7 +5369,7 @@
       </c>
       <c r="M89" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 088</t>
+          <t>Valve Repair scheduled or reactive task 088</t>
         </is>
       </c>
     </row>
@@ -5386,7 +5386,7 @@
       </c>
       <c r="C90" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D90" s="2" t="inlineStr">
@@ -5422,7 +5422,7 @@
       </c>
       <c r="M90" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 089</t>
+          <t>Pipe Replacement scheduled or reactive task 089</t>
         </is>
       </c>
     </row>
@@ -5439,7 +5439,7 @@
       </c>
       <c r="C91" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D91" s="2" t="inlineStr">
@@ -5475,7 +5475,7 @@
       </c>
       <c r="M91" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 090</t>
+          <t>Pipe Replacement scheduled or reactive task 090</t>
         </is>
       </c>
     </row>
@@ -5492,7 +5492,7 @@
       </c>
       <c r="C92" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D92" s="2" t="inlineStr">
@@ -5530,7 +5530,7 @@
       </c>
       <c r="M92" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 091</t>
+          <t>Pipe Replacement scheduled or reactive task 091</t>
         </is>
       </c>
     </row>
@@ -5547,7 +5547,7 @@
       </c>
       <c r="C93" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D93" s="2" t="inlineStr">
@@ -5585,7 +5585,7 @@
       </c>
       <c r="M93" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 092</t>
+          <t>Pipe Replacement scheduled or reactive task 092</t>
         </is>
       </c>
     </row>
@@ -5602,7 +5602,7 @@
       </c>
       <c r="C94" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D94" s="2" t="inlineStr">
@@ -5638,7 +5638,7 @@
       </c>
       <c r="M94" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 093</t>
+          <t>Pump Service scheduled or reactive task 093</t>
         </is>
       </c>
     </row>
@@ -5655,7 +5655,7 @@
       </c>
       <c r="C95" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D95" s="2" t="inlineStr">
@@ -5691,7 +5691,7 @@
       </c>
       <c r="M95" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 094</t>
+          <t>Pump Service scheduled or reactive task 094</t>
         </is>
       </c>
     </row>
@@ -5708,7 +5708,7 @@
       </c>
       <c r="C96" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D96" s="2" t="inlineStr">
@@ -5744,7 +5744,7 @@
       </c>
       <c r="M96" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 095</t>
+          <t>Pump Service scheduled or reactive task 095</t>
         </is>
       </c>
     </row>
@@ -5761,7 +5761,7 @@
       </c>
       <c r="C97" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D97" s="2" t="inlineStr">
@@ -5799,7 +5799,7 @@
       </c>
       <c r="M97" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 096</t>
+          <t>Pump Service scheduled or reactive task 096</t>
         </is>
       </c>
     </row>
@@ -5816,7 +5816,7 @@
       </c>
       <c r="C98" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D98" s="2" t="inlineStr">
@@ -5854,7 +5854,7 @@
       </c>
       <c r="M98" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 097</t>
+          <t>Meter Service scheduled or reactive task 097</t>
         </is>
       </c>
     </row>
@@ -5871,7 +5871,7 @@
       </c>
       <c r="C99" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D99" s="2" t="inlineStr">
@@ -5907,7 +5907,7 @@
       </c>
       <c r="M99" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 098</t>
+          <t>Meter Service scheduled or reactive task 098</t>
         </is>
       </c>
     </row>
@@ -5924,7 +5924,7 @@
       </c>
       <c r="C100" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D100" s="2" t="inlineStr">
@@ -5960,7 +5960,7 @@
       </c>
       <c r="M100" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 099</t>
+          <t>Meter Service scheduled or reactive task 099</t>
         </is>
       </c>
     </row>
@@ -5977,7 +5977,7 @@
       </c>
       <c r="C101" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D101" s="2" t="inlineStr">
@@ -6013,7 +6013,7 @@
       </c>
       <c r="M101" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 100</t>
+          <t>Meter Service scheduled or reactive task 100</t>
         </is>
       </c>
     </row>
@@ -6030,7 +6030,7 @@
       </c>
       <c r="C102" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D102" s="2" t="inlineStr">
@@ -6068,7 +6068,7 @@
       </c>
       <c r="M102" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 101</t>
+          <t>Leak Repair scheduled or reactive task 101</t>
         </is>
       </c>
     </row>
@@ -6085,7 +6085,7 @@
       </c>
       <c r="C103" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D103" s="2" t="inlineStr">
@@ -6123,7 +6123,7 @@
       </c>
       <c r="M103" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 102</t>
+          <t>Leak Repair scheduled or reactive task 102</t>
         </is>
       </c>
     </row>
@@ -6140,7 +6140,7 @@
       </c>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D104" s="2" t="inlineStr">
@@ -6176,7 +6176,7 @@
       </c>
       <c r="M104" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 103</t>
+          <t>Leak Repair scheduled or reactive task 103</t>
         </is>
       </c>
     </row>
@@ -6193,7 +6193,7 @@
       </c>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="D105" s="2" t="inlineStr">
@@ -6229,7 +6229,7 @@
       </c>
       <c r="M105" s="2" t="inlineStr">
         <is>
-          <t>HVAC scheduled or reactive task 104</t>
+          <t>Leak Repair scheduled or reactive task 104</t>
         </is>
       </c>
     </row>
@@ -6246,7 +6246,7 @@
       </c>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D106" s="2" t="inlineStr">
@@ -6282,7 +6282,7 @@
       </c>
       <c r="M106" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 105</t>
+          <t>Valve Repair scheduled or reactive task 105</t>
         </is>
       </c>
     </row>
@@ -6299,7 +6299,7 @@
       </c>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D107" s="2" t="inlineStr">
@@ -6337,7 +6337,7 @@
       </c>
       <c r="M107" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 106</t>
+          <t>Valve Repair scheduled or reactive task 106</t>
         </is>
       </c>
     </row>
@@ -6354,7 +6354,7 @@
       </c>
       <c r="C108" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D108" s="2" t="inlineStr">
@@ -6392,7 +6392,7 @@
       </c>
       <c r="M108" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 107</t>
+          <t>Valve Repair scheduled or reactive task 107</t>
         </is>
       </c>
     </row>
@@ -6409,7 +6409,7 @@
       </c>
       <c r="C109" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D109" s="2" t="inlineStr">
@@ -6445,7 +6445,7 @@
       </c>
       <c r="M109" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 108</t>
+          <t>Valve Repair scheduled or reactive task 108</t>
         </is>
       </c>
     </row>
@@ -6462,7 +6462,7 @@
       </c>
       <c r="C110" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D110" s="2" t="inlineStr">
@@ -6494,7 +6494,7 @@
       </c>
       <c r="M110" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 109</t>
+          <t>Pipe Replacement scheduled or reactive task 109</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6511,7 @@
       </c>
       <c r="C111" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D111" s="2" t="inlineStr">
@@ -6547,7 +6547,7 @@
       </c>
       <c r="M111" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 110</t>
+          <t>Pipe Replacement scheduled or reactive task 110</t>
         </is>
       </c>
     </row>
@@ -6564,7 +6564,7 @@
       </c>
       <c r="C112" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D112" s="2" t="inlineStr">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="M112" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 111</t>
+          <t>Pipe Replacement scheduled or reactive task 111</t>
         </is>
       </c>
     </row>
@@ -6619,7 +6619,7 @@
       </c>
       <c r="C113" s="2" t="inlineStr">
         <is>
-          <t>Plumbing</t>
+          <t>Pipe Replacement</t>
         </is>
       </c>
       <c r="D113" s="2" t="inlineStr">
@@ -6657,7 +6657,7 @@
       </c>
       <c r="M113" s="2" t="inlineStr">
         <is>
-          <t>Plumbing scheduled or reactive task 112</t>
+          <t>Pipe Replacement scheduled or reactive task 112</t>
         </is>
       </c>
     </row>
@@ -6674,7 +6674,7 @@
       </c>
       <c r="C114" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D114" s="2" t="inlineStr">
@@ -6710,7 +6710,7 @@
       </c>
       <c r="M114" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 113</t>
+          <t>Pump Service scheduled or reactive task 113</t>
         </is>
       </c>
     </row>
@@ -6727,7 +6727,7 @@
       </c>
       <c r="C115" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D115" s="2" t="inlineStr">
@@ -6763,7 +6763,7 @@
       </c>
       <c r="M115" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 114</t>
+          <t>Pump Service scheduled or reactive task 114</t>
         </is>
       </c>
     </row>
@@ -6780,7 +6780,7 @@
       </c>
       <c r="C116" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D116" s="2" t="inlineStr">
@@ -6816,7 +6816,7 @@
       </c>
       <c r="M116" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 115</t>
+          <t>Pump Service scheduled or reactive task 115</t>
         </is>
       </c>
     </row>
@@ -6833,7 +6833,7 @@
       </c>
       <c r="C117" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety</t>
+          <t>Pump Service</t>
         </is>
       </c>
       <c r="D117" s="2" t="inlineStr">
@@ -6871,7 +6871,7 @@
       </c>
       <c r="M117" s="2" t="inlineStr">
         <is>
-          <t>Fire Safety scheduled or reactive task 116</t>
+          <t>Pump Service scheduled or reactive task 116</t>
         </is>
       </c>
     </row>
@@ -6888,7 +6888,7 @@
       </c>
       <c r="C118" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D118" s="2" t="inlineStr">
@@ -6926,7 +6926,7 @@
       </c>
       <c r="M118" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 117</t>
+          <t>Meter Service scheduled or reactive task 117</t>
         </is>
       </c>
     </row>
@@ -6943,7 +6943,7 @@
       </c>
       <c r="C119" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D119" s="2" t="inlineStr">
@@ -6979,7 +6979,7 @@
       </c>
       <c r="M119" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 118</t>
+          <t>Meter Service scheduled or reactive task 118</t>
         </is>
       </c>
     </row>
@@ -6996,7 +6996,7 @@
       </c>
       <c r="C120" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D120" s="2" t="inlineStr">
@@ -7032,7 +7032,7 @@
       </c>
       <c r="M120" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 119</t>
+          <t>Meter Service scheduled or reactive task 119</t>
         </is>
       </c>
     </row>
@@ -7049,7 +7049,7 @@
       </c>
       <c r="C121" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D121" s="2" t="inlineStr">
@@ -7085,7 +7085,7 @@
       </c>
       <c r="M121" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 120</t>
+          <t>Meter Service scheduled or reactive task 120</t>
         </is>
       </c>
     </row>
@@ -7102,7 +7102,7 @@
       </c>
       <c r="C122" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="D122" s="2" t="inlineStr">
@@ -7138,7 +7138,7 @@
       </c>
       <c r="M122" s="2" t="inlineStr">
         <is>
-          <t>Electrical scheduled or reactive task 005</t>
+          <t>Valve Repair scheduled or reactive task 005</t>
         </is>
       </c>
     </row>
@@ -7155,7 +7155,7 @@
       </c>
       <c r="C123" s="2" t="inlineStr">
         <is>
-          <t>General Repair</t>
+          <t>Meter Service</t>
         </is>
       </c>
       <c r="D123" s="2" t="inlineStr">
@@ -7191,7 +7191,7 @@
       </c>
       <c r="M123" s="2" t="inlineStr">
         <is>
-          <t>General Repair scheduled or reactive task 020</t>
+          <t>Meter Service scheduled or reactive task 020</t>
         </is>
       </c>
     </row>
@@ -7249,7 +7249,7 @@
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="C2" s="2" t="n">
@@ -7269,7 +7269,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="C3" s="2" t="n">
@@ -7289,7 +7289,7 @@
       </c>
       <c r="B4" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="C4" s="2" t="n">
@@ -7309,7 +7309,7 @@
       </c>
       <c r="B5" s="2" t="inlineStr">
         <is>
-          <t>HVAC</t>
+          <t>Leak Repair</t>
         </is>
       </c>
       <c r="C5" s="2" t="n">
@@ -7329,7 +7329,7 @@
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="C6" s="2" t="n">
@@ -7349,7 +7349,7 @@
       </c>
       <c r="B7" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="C7" s="2" t="n">
@@ -7369,7 +7369,7 @@
       </c>
       <c r="B8" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="C8" s="2" t="n">
@@ -7389,7 +7389,7 @@
       </c>
       <c r="B9" s="2" t="inlineStr">
         <is>
-          <t>Electrical</t>
+          <t>Valve Repair</t>
         </is>
       </c>
       <c r="C9" s="2" t="n">
@@ -7595,7 +7595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F5"/>
+  <dimension ref="A1:F7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -7641,33 +7641,51 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
+          <t>Step 1</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>EXCEL - CHAT ONLY</t>
+        </is>
+      </c>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>EXCEL - CHAT ONLY:
+Read About_This_Data and Control for Northstar Water Services. Explain what one water-pipe service work order represents, the reporting date, the five job categories and how current owners differ from proposed owners. Do not edit or infer customer impacts.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="2" t="inlineStr">
+        <is>
           <t>Step 2</t>
         </is>
       </c>
-      <c r="B2" s="2" t="inlineStr">
+      <c r="B3" s="2" t="inlineStr">
         <is>
           <t>EXCEL - CHAT ONLY</t>
         </is>
       </c>
-      <c r="C2" s="2" t="inlineStr">
+      <c r="C3" s="2" t="inlineStr">
         <is>
           <t>EXCEL - CHAT ONLY:
 Inspect tblWorkOrders. Report row count, duplicate Work_Order_ID values, category spelling variants and missing Assigned_To. Do not edit. Treat 2026-09-30 as the fixed reporting date.</t>
         </is>
       </c>
     </row>
-    <row r="3">
-      <c r="A3" s="2" t="inlineStr">
+    <row r="4">
+      <c r="A4" s="2" t="inlineStr">
         <is>
           <t>Step 3</t>
         </is>
       </c>
-      <c r="B3" s="2" t="inlineStr">
+      <c r="B4" s="2" t="inlineStr">
         <is>
           <t>EXCEL - PLAN</t>
         </is>
       </c>
-      <c r="C3" s="2" t="inlineStr">
+      <c r="C4" s="2" t="inlineStr">
         <is>
           <t>EXCEL - PLAN:
 Plan to retain an untouched Raw_Export copy, remove only exact duplicate records by Work_Order_ID, and standardise category spelling in tblWorkOrders. Keep dates, statuses and assignments. Ask if two records with one ID differ.
@@ -7676,39 +7694,57 @@
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="2" t="inlineStr">
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
         <is>
           <t>Step 4</t>
         </is>
       </c>
-      <c r="B4" s="2" t="inlineStr">
+      <c r="B5" s="2" t="inlineStr">
         <is>
           <t>EXCEL - ALLOW EDITING</t>
         </is>
       </c>
-      <c r="C4" s="2" t="inlineStr">
+      <c r="C5" s="2" t="inlineStr">
         <is>
           <t>EXCEL - ALLOW EDITING:
 In Checks calculate total rows, closed, cancelled, backlog, overdue backlog, unassigned backlog and total Cost_SGD for tblWorkOrders. Use Control!B2 as reporting date. Define backlog as Status neither Closed nor Cancelled. Add the identity total = closed + cancelled + backlog. Do not change source data.</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="2" t="inlineStr">
+    <row r="6">
+      <c r="A6" s="2" t="inlineStr">
         <is>
           <t>Step 5</t>
         </is>
       </c>
-      <c r="B5" s="2" t="inlineStr">
+      <c r="B6" s="2" t="inlineStr">
         <is>
           <t>WORD COPILOT</t>
         </is>
       </c>
-      <c r="C5" s="2" t="inlineStr">
+      <c r="C6" s="2" t="inlineStr">
         <is>
           <t>WORD COPILOT:
 Draft a one-page Northstar operations brief from the verified evidence supplied here. Include reporting scope/date, backlog and overdue findings, current assignment issues, proposed next actions and open questions. Keep observed facts separate from proposals. Preserve numbers and definitions. Use UNKNOWN for causes, approvals or capacity decisions not evidenced.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Step 6</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>WORD COPILOT</t>
+        </is>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>WORD COPILOT:
+Audit this Northstar Water Services operations brief against the verified evidence table I supply. Return a discrepancy list for counts, cost, reporting scope, overdue definition and assignment claims. Identify missing source links as UNKNOWN. Do not change facts or approve work.</t>
         </is>
       </c>
     </row>

</xml_diff>